<commit_message>
Estadisticos Final 10 Mañana
</commit_message>
<xml_diff>
--- a/DetalleXDocente20241.xlsx
+++ b/DetalleXDocente20241.xlsx
@@ -5716,13 +5716,13 @@
         <v>24</v>
       </c>
       <c r="E151">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F151">
         <v>1</v>
       </c>
       <c r="G151" s="1">
-        <v>91.7</v>
+        <v>95.8</v>
       </c>
       <c r="H151" s="1">
         <v>4.2</v>
@@ -5731,10 +5731,10 @@
         <v>8.5</v>
       </c>
       <c r="J151">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K151" s="1">
-        <v>4.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="152" spans="1:11">
@@ -5748,13 +5748,13 @@
         <v>85</v>
       </c>
       <c r="E152">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F152">
         <v>11</v>
       </c>
       <c r="G152" s="1">
-        <v>85.90000000000001</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="H152" s="1">
         <v>12.9</v>
@@ -5763,10 +5763,10 @@
         <v>7.6</v>
       </c>
       <c r="J152">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K152" s="1">
-        <v>1.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="153" spans="1:11">
@@ -15731,13 +15731,13 @@
         <v>24</v>
       </c>
       <c r="E151">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F151">
         <v>0</v>
       </c>
       <c r="G151" s="1">
-        <v>95.8</v>
+        <v>100</v>
       </c>
       <c r="H151" s="1">
         <v>0</v>
@@ -15746,10 +15746,10 @@
         <v>8.699999999999999</v>
       </c>
       <c r="J151">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K151" s="1">
-        <v>4.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="152" spans="1:11">
@@ -15763,13 +15763,13 @@
         <v>85</v>
       </c>
       <c r="E152">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F152">
         <v>10</v>
       </c>
       <c r="G152" s="1">
-        <v>87.09999999999999</v>
+        <v>88.2</v>
       </c>
       <c r="H152" s="1">
         <v>11.8</v>
@@ -15778,10 +15778,10 @@
         <v>8</v>
       </c>
       <c r="J152">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K152" s="1">
-        <v>1.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="153" spans="1:11">
@@ -21325,25 +21325,25 @@
         <v>39</v>
       </c>
       <c r="E15">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="F15">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G15" s="1">
-        <v>100</v>
+        <v>89.7</v>
       </c>
       <c r="H15" s="1">
-        <v>0</v>
+        <v>10.3</v>
       </c>
       <c r="I15" s="2">
-        <v>7.7</v>
+        <v>7.5</v>
       </c>
       <c r="J15">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="K15" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -21360,25 +21360,25 @@
         <v>34</v>
       </c>
       <c r="E16">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G16" s="1">
-        <v>91.2</v>
+        <v>88.2</v>
       </c>
       <c r="H16" s="1">
-        <v>8.800000000000001</v>
+        <v>11.8</v>
       </c>
       <c r="I16" s="2">
-        <v>7.7</v>
+        <v>7.4</v>
       </c>
       <c r="J16">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="K16" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:11">
@@ -21395,25 +21395,25 @@
         <v>33</v>
       </c>
       <c r="E17">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="F17">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G17" s="1">
-        <v>81.8</v>
+        <v>72.7</v>
       </c>
       <c r="H17" s="1">
-        <v>18.2</v>
+        <v>27.3</v>
       </c>
       <c r="I17" s="2">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
       <c r="J17">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="K17" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -21430,25 +21430,25 @@
         <v>23</v>
       </c>
       <c r="E18">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="F18">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G18" s="1">
-        <v>100</v>
+        <v>78.3</v>
       </c>
       <c r="H18" s="1">
-        <v>0</v>
+        <v>21.7</v>
       </c>
       <c r="I18" s="2">
-        <v>7.7</v>
+        <v>7.2</v>
       </c>
       <c r="J18">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="K18" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -21465,25 +21465,25 @@
         <v>19</v>
       </c>
       <c r="E19">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G19" s="1">
-        <v>100</v>
+        <v>94.7</v>
       </c>
       <c r="H19" s="1">
-        <v>0</v>
+        <v>5.3</v>
       </c>
       <c r="I19" s="2">
-        <v>8.6</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="J19">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="K19" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:11">
@@ -21515,10 +21515,10 @@
         <v>9.300000000000001</v>
       </c>
       <c r="J20">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K20" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:11">
@@ -21532,25 +21532,25 @@
         <v>158</v>
       </c>
       <c r="E21">
-        <v>149</v>
+        <v>135</v>
       </c>
       <c r="F21">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="G21" s="1">
-        <v>94.3</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="H21" s="1">
-        <v>5.7</v>
+        <v>14.6</v>
       </c>
       <c r="I21" s="2">
-        <v>8</v>
+        <v>7.8</v>
       </c>
       <c r="J21">
-        <v>158</v>
+        <v>0</v>
       </c>
       <c r="K21" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:11">
@@ -21567,25 +21567,25 @@
         <v>36</v>
       </c>
       <c r="E22">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F22">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G22" s="1">
-        <v>94.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="H22" s="1">
-        <v>5.6</v>
+        <v>0</v>
       </c>
       <c r="I22" s="2">
-        <v>7.8</v>
+        <v>7.9</v>
       </c>
       <c r="J22">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="K22" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:11">
@@ -21602,25 +21602,25 @@
         <v>36</v>
       </c>
       <c r="E23">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="F23">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G23" s="1">
-        <v>88.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="H23" s="1">
-        <v>11.1</v>
+        <v>0</v>
       </c>
       <c r="I23" s="2">
-        <v>7.8</v>
+        <v>8.1</v>
       </c>
       <c r="J23">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="K23" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:11">
@@ -21637,25 +21637,25 @@
         <v>37</v>
       </c>
       <c r="E24">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F24">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G24" s="1">
-        <v>97.3</v>
+        <v>100</v>
       </c>
       <c r="H24" s="1">
-        <v>2.7</v>
+        <v>0</v>
       </c>
       <c r="I24" s="2">
         <v>8.699999999999999</v>
       </c>
       <c r="J24">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="K24" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:11">
@@ -21672,25 +21672,25 @@
         <v>37</v>
       </c>
       <c r="E25">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F25">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G25" s="1">
-        <v>94.59999999999999</v>
+        <v>100</v>
       </c>
       <c r="H25" s="1">
-        <v>5.4</v>
+        <v>0</v>
       </c>
       <c r="I25" s="2">
-        <v>8.6</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J25">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="K25" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:11">
@@ -21704,25 +21704,25 @@
         <v>146</v>
       </c>
       <c r="E26">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="F26">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="G26" s="1">
-        <v>93.8</v>
+        <v>100</v>
       </c>
       <c r="H26" s="1">
-        <v>6.2</v>
+        <v>0</v>
       </c>
       <c r="I26" s="2">
-        <v>8.199999999999999</v>
+        <v>8.4</v>
       </c>
       <c r="J26">
-        <v>146</v>
+        <v>0</v>
       </c>
       <c r="K26" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:11">
@@ -22048,25 +22048,25 @@
         <v>34</v>
       </c>
       <c r="E36">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="F36">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="G36" s="1">
-        <v>52.9</v>
+        <v>85.3</v>
       </c>
       <c r="H36" s="1">
-        <v>47.1</v>
+        <v>14.7</v>
       </c>
       <c r="I36" s="2">
-        <v>6.5</v>
+        <v>6.9</v>
       </c>
       <c r="J36">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="K36" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:11">
@@ -22118,25 +22118,25 @@
         <v>23</v>
       </c>
       <c r="E38">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F38">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G38" s="1">
-        <v>82.59999999999999</v>
+        <v>95.7</v>
       </c>
       <c r="H38" s="1">
-        <v>17.4</v>
+        <v>4.3</v>
       </c>
       <c r="I38" s="2">
-        <v>7.6</v>
+        <v>7.7</v>
       </c>
       <c r="J38">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="K38" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:11">
@@ -22185,25 +22185,25 @@
         <v>149</v>
       </c>
       <c r="E40">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="F40">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="G40" s="1">
-        <v>79.90000000000001</v>
+        <v>89.3</v>
       </c>
       <c r="H40" s="1">
-        <v>20.1</v>
+        <v>10.7</v>
       </c>
       <c r="I40" s="2">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
       <c r="J40">
-        <v>57</v>
+        <v>0</v>
       </c>
       <c r="K40" s="1">
-        <v>38.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:11">
@@ -22608,13 +22608,13 @@
         <v>17.5</v>
       </c>
       <c r="I52" s="2">
-        <v>6.9</v>
+        <v>6.5</v>
       </c>
       <c r="J52">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="K52" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53" spans="1:11">
@@ -22631,25 +22631,25 @@
         <v>34</v>
       </c>
       <c r="E53">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="F53">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G53" s="1">
-        <v>67.59999999999999</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="H53" s="1">
-        <v>32.4</v>
+        <v>17.6</v>
       </c>
       <c r="I53" s="2">
-        <v>6.7</v>
+        <v>6.5</v>
       </c>
       <c r="J53">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="K53" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54" spans="1:11">
@@ -22666,25 +22666,25 @@
         <v>33</v>
       </c>
       <c r="E54">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F54">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G54" s="1">
-        <v>69.7</v>
+        <v>75.8</v>
       </c>
       <c r="H54" s="1">
-        <v>30.3</v>
+        <v>24.2</v>
       </c>
       <c r="I54" s="2">
-        <v>6.7</v>
+        <v>6.6</v>
       </c>
       <c r="J54">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="K54" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55" spans="1:11">
@@ -22736,25 +22736,25 @@
         <v>19</v>
       </c>
       <c r="E56">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F56">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G56" s="1">
-        <v>78.90000000000001</v>
+        <v>84.2</v>
       </c>
       <c r="H56" s="1">
-        <v>21.1</v>
+        <v>15.8</v>
       </c>
       <c r="I56" s="2">
-        <v>7.1</v>
+        <v>6.8</v>
       </c>
       <c r="J56">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="K56" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="57" spans="1:11">
@@ -22803,25 +22803,25 @@
         <v>170</v>
       </c>
       <c r="E58">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="F58">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="G58" s="1">
-        <v>68.2</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="H58" s="1">
-        <v>31.8</v>
+        <v>27.1</v>
       </c>
       <c r="I58" s="2">
-        <v>6.6</v>
+        <v>6.4</v>
       </c>
       <c r="J58">
-        <v>170</v>
+        <v>44</v>
       </c>
       <c r="K58" s="1">
-        <v>100</v>
+        <v>25.9</v>
       </c>
     </row>
     <row r="59" spans="1:11">
@@ -23364,25 +23364,25 @@
         <v>25</v>
       </c>
       <c r="E82">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F82">
+        <v>1</v>
+      </c>
+      <c r="G82" s="1">
+        <v>96</v>
+      </c>
+      <c r="H82" s="1">
         <v>4</v>
       </c>
-      <c r="G82" s="1">
-        <v>84</v>
-      </c>
-      <c r="H82" s="1">
-        <v>16</v>
-      </c>
       <c r="I82" s="2">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
       <c r="J82">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="K82" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="83" spans="1:11">
@@ -23399,25 +23399,25 @@
         <v>28</v>
       </c>
       <c r="E83">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F83">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G83" s="1">
-        <v>89.3</v>
+        <v>85.7</v>
       </c>
       <c r="H83" s="1">
-        <v>10.7</v>
+        <v>14.3</v>
       </c>
       <c r="I83" s="2">
         <v>7.6</v>
       </c>
       <c r="J83">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="K83" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="84" spans="1:11">
@@ -23431,25 +23431,25 @@
         <v>53</v>
       </c>
       <c r="E84">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F84">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G84" s="1">
-        <v>86.8</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="H84" s="1">
-        <v>13.2</v>
+        <v>9.4</v>
       </c>
       <c r="I84" s="2">
         <v>7.4</v>
       </c>
       <c r="J84">
-        <v>53</v>
+        <v>0</v>
       </c>
       <c r="K84" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85" spans="1:11">
@@ -23673,25 +23673,25 @@
         <v>21</v>
       </c>
       <c r="E91">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F91">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G91" s="1">
-        <v>61.9</v>
+        <v>85.7</v>
       </c>
       <c r="H91" s="1">
-        <v>38.1</v>
+        <v>14.3</v>
       </c>
       <c r="I91" s="2">
-        <v>5.9</v>
+        <v>6.1</v>
       </c>
       <c r="J91">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="K91" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92" spans="1:11">
@@ -23708,25 +23708,25 @@
         <v>25</v>
       </c>
       <c r="E92">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F92">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G92" s="1">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="H92" s="1">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="I92" s="2">
-        <v>7.4</v>
+        <v>7.3</v>
       </c>
       <c r="J92">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="K92" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="93" spans="1:11">
@@ -23755,13 +23755,13 @@
         <v>4.8</v>
       </c>
       <c r="I93" s="2">
-        <v>8</v>
+        <v>7.6</v>
       </c>
       <c r="J93">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="K93" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="94" spans="1:11">
@@ -23845,25 +23845,25 @@
         <v>109</v>
       </c>
       <c r="E96">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="F96">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="G96" s="1">
-        <v>80.7</v>
+        <v>87.2</v>
       </c>
       <c r="H96" s="1">
-        <v>19.3</v>
+        <v>12.8</v>
       </c>
       <c r="I96" s="2">
-        <v>7.3</v>
+        <v>7.2</v>
       </c>
       <c r="J96">
-        <v>108</v>
+        <v>41</v>
       </c>
       <c r="K96" s="1">
-        <v>99.09999999999999</v>
+        <v>37.6</v>
       </c>
     </row>
     <row r="97" spans="1:11">
@@ -23880,25 +23880,25 @@
         <v>40</v>
       </c>
       <c r="E97">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F97">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G97" s="1">
-        <v>97.5</v>
+        <v>95</v>
       </c>
       <c r="H97" s="1">
-        <v>2.5</v>
+        <v>5</v>
       </c>
       <c r="I97" s="2">
-        <v>7.2</v>
+        <v>7.4</v>
       </c>
       <c r="J97">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="K97" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="98" spans="1:11">
@@ -23915,25 +23915,25 @@
         <v>41</v>
       </c>
       <c r="E98">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="F98">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G98" s="1">
-        <v>87.8</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="H98" s="1">
-        <v>12.2</v>
+        <v>2.4</v>
       </c>
       <c r="I98" s="2">
         <v>6.8</v>
       </c>
       <c r="J98">
-        <v>41</v>
+        <v>0</v>
       </c>
       <c r="K98" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="99" spans="1:11">
@@ -23950,25 +23950,25 @@
         <v>48</v>
       </c>
       <c r="E99">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="F99">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="G99" s="1">
-        <v>83.3</v>
+        <v>100</v>
       </c>
       <c r="H99" s="1">
-        <v>16.7</v>
+        <v>0</v>
       </c>
       <c r="I99" s="2">
-        <v>7</v>
+        <v>7.4</v>
       </c>
       <c r="J99">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="K99" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="100" spans="1:11">
@@ -24055,25 +24055,25 @@
         <v>33</v>
       </c>
       <c r="E102">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F102">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G102" s="1">
-        <v>93.90000000000001</v>
+        <v>97</v>
       </c>
       <c r="H102" s="1">
-        <v>6.1</v>
+        <v>3</v>
       </c>
       <c r="I102" s="2">
-        <v>7.3</v>
+        <v>7.5</v>
       </c>
       <c r="J102">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="K102" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="103" spans="1:11">
@@ -24087,25 +24087,25 @@
         <v>235</v>
       </c>
       <c r="E103">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="F103">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="G103" s="1">
-        <v>91.5</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="H103" s="1">
-        <v>8.5</v>
+        <v>3.4</v>
       </c>
       <c r="I103" s="2">
-        <v>7.1</v>
+        <v>7.3</v>
       </c>
       <c r="J103">
-        <v>235</v>
+        <v>73</v>
       </c>
       <c r="K103" s="1">
-        <v>100</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="104" spans="1:11">
@@ -24312,10 +24312,10 @@
         <v>9.300000000000001</v>
       </c>
       <c r="J109">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="K109" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="110" spans="1:11">
@@ -24379,10 +24379,10 @@
         <v>8.6</v>
       </c>
       <c r="J111">
-        <v>76</v>
+        <v>40</v>
       </c>
       <c r="K111" s="1">
-        <v>31.8</v>
+        <v>16.7</v>
       </c>
     </row>
     <row r="112" spans="1:11">
@@ -24399,25 +24399,25 @@
         <v>33</v>
       </c>
       <c r="E112">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F112">
+        <v>1</v>
+      </c>
+      <c r="G112" s="1">
+        <v>97</v>
+      </c>
+      <c r="H112" s="1">
         <v>3</v>
       </c>
-      <c r="G112" s="1">
-        <v>90.90000000000001</v>
-      </c>
-      <c r="H112" s="1">
-        <v>9.1</v>
-      </c>
       <c r="I112" s="2">
-        <v>8.1</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="J112">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="K112" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="113" spans="1:11">
@@ -24434,25 +24434,25 @@
         <v>21</v>
       </c>
       <c r="E113">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F113">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G113" s="1">
-        <v>85.7</v>
+        <v>90.5</v>
       </c>
       <c r="H113" s="1">
-        <v>14.3</v>
+        <v>9.5</v>
       </c>
       <c r="I113" s="2">
-        <v>7.5</v>
+        <v>7.8</v>
       </c>
       <c r="J113">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="K113" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="114" spans="1:11">
@@ -24469,25 +24469,25 @@
         <v>25</v>
       </c>
       <c r="E114">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F114">
+        <v>1</v>
+      </c>
+      <c r="G114" s="1">
+        <v>96</v>
+      </c>
+      <c r="H114" s="1">
         <v>4</v>
       </c>
-      <c r="G114" s="1">
-        <v>84</v>
-      </c>
-      <c r="H114" s="1">
-        <v>16</v>
-      </c>
       <c r="I114" s="2">
-        <v>7.7</v>
+        <v>7.5</v>
       </c>
       <c r="J114">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="K114" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="115" spans="1:11">
@@ -24504,25 +24504,25 @@
         <v>19</v>
       </c>
       <c r="E115">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F115">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G115" s="1">
-        <v>84.2</v>
+        <v>94.7</v>
       </c>
       <c r="H115" s="1">
-        <v>15.8</v>
+        <v>5.3</v>
       </c>
       <c r="I115" s="2">
-        <v>8.1</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="J115">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="K115" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="116" spans="1:11">
@@ -24571,25 +24571,25 @@
         <v>119</v>
       </c>
       <c r="E117">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="F117">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="G117" s="1">
-        <v>88.2</v>
+        <v>95</v>
       </c>
       <c r="H117" s="1">
-        <v>11.8</v>
+        <v>5</v>
       </c>
       <c r="I117" s="2">
-        <v>7.9</v>
+        <v>8</v>
       </c>
       <c r="J117">
-        <v>98</v>
+        <v>0</v>
       </c>
       <c r="K117" s="1">
-        <v>82.40000000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="118" spans="1:11">
@@ -25239,13 +25239,13 @@
         <v>0</v>
       </c>
       <c r="I136" s="2">
-        <v>8</v>
+        <v>7.9</v>
       </c>
       <c r="J136">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="K136" s="1">
-        <v>66.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="137" spans="1:11">
@@ -25309,13 +25309,13 @@
         <v>0</v>
       </c>
       <c r="I138" s="2">
-        <v>7.6</v>
+        <v>8</v>
       </c>
       <c r="J138">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="K138" s="1">
-        <v>100</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="139" spans="1:11">
@@ -25332,25 +25332,25 @@
         <v>22</v>
       </c>
       <c r="E139">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F139">
+        <v>0</v>
+      </c>
+      <c r="G139" s="1">
+        <v>95.5</v>
+      </c>
+      <c r="H139" s="1">
+        <v>0</v>
+      </c>
+      <c r="I139" s="2">
+        <v>6.9</v>
+      </c>
+      <c r="J139">
         <v>1</v>
       </c>
-      <c r="G139" s="1">
-        <v>90.90000000000001</v>
-      </c>
-      <c r="H139" s="1">
+      <c r="K139" s="1">
         <v>4.5</v>
-      </c>
-      <c r="I139" s="2">
-        <v>7.5</v>
-      </c>
-      <c r="J139">
-        <v>22</v>
-      </c>
-      <c r="K139" s="1">
-        <v>100</v>
       </c>
     </row>
     <row r="140" spans="1:11">
@@ -25367,25 +25367,25 @@
         <v>28</v>
       </c>
       <c r="E140">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F140">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G140" s="1">
-        <v>96.40000000000001</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="H140" s="1">
-        <v>3.6</v>
+        <v>17.9</v>
       </c>
       <c r="I140" s="2">
-        <v>8.300000000000001</v>
+        <v>8</v>
       </c>
       <c r="J140">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="K140" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="141" spans="1:11">
@@ -25399,25 +25399,25 @@
         <v>127</v>
       </c>
       <c r="E141">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="F141">
+        <v>5</v>
+      </c>
+      <c r="G141" s="1">
+        <v>94.5</v>
+      </c>
+      <c r="H141" s="1">
+        <v>3.9</v>
+      </c>
+      <c r="I141" s="2">
+        <v>7.8</v>
+      </c>
+      <c r="J141">
         <v>2</v>
       </c>
-      <c r="G141" s="1">
-        <v>96.90000000000001</v>
-      </c>
-      <c r="H141" s="1">
+      <c r="K141" s="1">
         <v>1.6</v>
-      </c>
-      <c r="I141" s="2">
-        <v>7.9</v>
-      </c>
-      <c r="J141">
-        <v>95</v>
-      </c>
-      <c r="K141" s="1">
-        <v>74.8</v>
       </c>
     </row>
     <row r="142" spans="1:11">
@@ -25641,25 +25641,25 @@
         <v>21</v>
       </c>
       <c r="E148">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F148">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G148" s="1">
-        <v>71.40000000000001</v>
+        <v>85.7</v>
       </c>
       <c r="H148" s="1">
-        <v>28.6</v>
+        <v>14.3</v>
       </c>
       <c r="I148" s="2">
-        <v>6.9</v>
+        <v>7</v>
       </c>
       <c r="J148">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="K148" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="149" spans="1:11">
@@ -25676,25 +25676,25 @@
         <v>19</v>
       </c>
       <c r="E149">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F149">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G149" s="1">
-        <v>89.5</v>
+        <v>94.7</v>
       </c>
       <c r="H149" s="1">
-        <v>10.5</v>
+        <v>5.3</v>
       </c>
       <c r="I149" s="2">
-        <v>8.300000000000001</v>
+        <v>8</v>
       </c>
       <c r="J149">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="K149" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="150" spans="1:11">
@@ -25711,25 +25711,25 @@
         <v>21</v>
       </c>
       <c r="E150">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F150">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G150" s="1">
-        <v>90.5</v>
+        <v>95.2</v>
       </c>
       <c r="H150" s="1">
-        <v>9.5</v>
+        <v>4.8</v>
       </c>
       <c r="I150" s="2">
-        <v>8.199999999999999</v>
+        <v>8</v>
       </c>
       <c r="J150">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="K150" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="151" spans="1:11">
@@ -25746,25 +25746,25 @@
         <v>24</v>
       </c>
       <c r="E151">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F151">
         <v>0</v>
       </c>
       <c r="G151" s="1">
-        <v>95.8</v>
+        <v>100</v>
       </c>
       <c r="H151" s="1">
         <v>0</v>
       </c>
       <c r="I151" s="2">
-        <v>8.9</v>
+        <v>8.6</v>
       </c>
       <c r="J151">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="K151" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="152" spans="1:11">
@@ -25778,25 +25778,25 @@
         <v>85</v>
       </c>
       <c r="E152">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="F152">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G152" s="1">
-        <v>87.09999999999999</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="H152" s="1">
-        <v>11.8</v>
+        <v>5.9</v>
       </c>
       <c r="I152" s="2">
-        <v>8.1</v>
+        <v>7.9</v>
       </c>
       <c r="J152">
-        <v>85</v>
+        <v>0</v>
       </c>
       <c r="K152" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="153" spans="1:11">
@@ -26755,13 +26755,13 @@
         <v>20.8</v>
       </c>
       <c r="I180" s="2">
-        <v>7.7</v>
+        <v>7.9</v>
       </c>
       <c r="J180">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="K180" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="181" spans="1:11">
@@ -26778,25 +26778,25 @@
         <v>36</v>
       </c>
       <c r="E181">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="F181">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G181" s="1">
-        <v>88.90000000000001</v>
+        <v>97.2</v>
       </c>
       <c r="H181" s="1">
-        <v>11.1</v>
+        <v>2.8</v>
       </c>
       <c r="I181" s="2">
-        <v>8</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="J181">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="K181" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="182" spans="1:11">
@@ -26813,25 +26813,25 @@
         <v>28</v>
       </c>
       <c r="E182">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F182">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G182" s="1">
-        <v>92.90000000000001</v>
+        <v>96.40000000000001</v>
       </c>
       <c r="H182" s="1">
-        <v>7.1</v>
+        <v>3.6</v>
       </c>
       <c r="I182" s="2">
-        <v>8.300000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="J182">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="K182" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="183" spans="1:11">
@@ -26848,25 +26848,25 @@
         <v>35</v>
       </c>
       <c r="E183">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="F183">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G183" s="1">
-        <v>88.59999999999999</v>
+        <v>100</v>
       </c>
       <c r="H183" s="1">
-        <v>11.4</v>
+        <v>0</v>
       </c>
       <c r="I183" s="2">
-        <v>8.5</v>
+        <v>8.9</v>
       </c>
       <c r="J183">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="K183" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="184" spans="1:11">
@@ -26883,25 +26883,25 @@
         <v>24</v>
       </c>
       <c r="E184">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="F184">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G184" s="1">
-        <v>70.8</v>
+        <v>100</v>
       </c>
       <c r="H184" s="1">
-        <v>29.2</v>
+        <v>0</v>
       </c>
       <c r="I184" s="2">
-        <v>7.2</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="J184">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="K184" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="185" spans="1:11">
@@ -26930,13 +26930,13 @@
         <v>2.7</v>
       </c>
       <c r="I185" s="2">
-        <v>8.800000000000001</v>
+        <v>9</v>
       </c>
       <c r="J185">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="K185" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="186" spans="1:11">
@@ -26950,25 +26950,25 @@
         <v>184</v>
       </c>
       <c r="E186">
-        <v>161</v>
+        <v>176</v>
       </c>
       <c r="F186">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="G186" s="1">
-        <v>87.5</v>
+        <v>95.7</v>
       </c>
       <c r="H186" s="1">
-        <v>12.5</v>
+        <v>4.3</v>
       </c>
       <c r="I186" s="2">
-        <v>8.1</v>
+        <v>8.5</v>
       </c>
       <c r="J186">
-        <v>184</v>
+        <v>0</v>
       </c>
       <c r="K186" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="187" spans="1:11">
@@ -28574,25 +28574,25 @@
         <v>28</v>
       </c>
       <c r="E233">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F233">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G233" s="1">
-        <v>75</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="H233" s="1">
-        <v>25</v>
+        <v>17.9</v>
       </c>
       <c r="I233" s="2">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="J233">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="K233" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="234" spans="1:11">
@@ -28609,25 +28609,25 @@
         <v>18</v>
       </c>
       <c r="E234">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F234">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G234" s="1">
-        <v>83.3</v>
+        <v>100</v>
       </c>
       <c r="H234" s="1">
-        <v>16.7</v>
+        <v>0</v>
       </c>
       <c r="I234" s="2">
-        <v>7.3</v>
+        <v>7.4</v>
       </c>
       <c r="J234">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="K234" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="235" spans="1:11">
@@ -28656,13 +28656,13 @@
         <v>0</v>
       </c>
       <c r="I235" s="2">
-        <v>8.300000000000001</v>
+        <v>8</v>
       </c>
       <c r="J235">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="K235" s="1">
-        <v>100</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="236" spans="1:11">
@@ -28676,25 +28676,25 @@
         <v>91</v>
       </c>
       <c r="E236">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="F236">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="G236" s="1">
-        <v>82.40000000000001</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="H236" s="1">
-        <v>15.4</v>
+        <v>9.9</v>
       </c>
       <c r="I236" s="2">
         <v>7</v>
       </c>
       <c r="J236">
-        <v>71</v>
+        <v>2</v>
       </c>
       <c r="K236" s="1">
-        <v>78</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="237" spans="1:11">
@@ -29067,10 +29067,10 @@
         <v>9.300000000000001</v>
       </c>
       <c r="J247">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="K247" s="1">
-        <v>36.4</v>
+        <v>9.1</v>
       </c>
     </row>
     <row r="248" spans="1:11">
@@ -29099,10 +29099,10 @@
         <v>9.300000000000001</v>
       </c>
       <c r="J248">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="K248" s="1">
-        <v>36.4</v>
+        <v>9.1</v>
       </c>
     </row>
     <row r="249" spans="1:11">
@@ -29632,25 +29632,25 @@
         <v>40</v>
       </c>
       <c r="E264">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="F264">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="G264" s="1">
-        <v>45</v>
+        <v>72.5</v>
       </c>
       <c r="H264" s="1">
-        <v>55</v>
+        <v>27.5</v>
       </c>
       <c r="I264" s="2">
-        <v>5.8</v>
+        <v>6.1</v>
       </c>
       <c r="J264">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="K264" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="265" spans="1:11">
@@ -29664,25 +29664,25 @@
         <v>40</v>
       </c>
       <c r="E265">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="F265">
-        <v>22</v>
+        <v>11</v>
       </c>
       <c r="G265" s="1">
-        <v>45</v>
+        <v>72.5</v>
       </c>
       <c r="H265" s="1">
-        <v>55</v>
+        <v>27.5</v>
       </c>
       <c r="I265" s="2">
-        <v>5.8</v>
+        <v>6.1</v>
       </c>
       <c r="J265">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="K265" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="266" spans="1:11">
@@ -29976,25 +29976,25 @@
         <v>48</v>
       </c>
       <c r="E274">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="F274">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G274" s="1">
-        <v>85.40000000000001</v>
+        <v>95.8</v>
       </c>
       <c r="H274" s="1">
-        <v>14.6</v>
+        <v>4.2</v>
       </c>
       <c r="I274" s="2">
-        <v>8</v>
+        <v>8.1</v>
       </c>
       <c r="J274">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="K274" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="275" spans="1:11">
@@ -30058,13 +30058,13 @@
         <v>6.1</v>
       </c>
       <c r="I276" s="2">
-        <v>8.699999999999999</v>
+        <v>8.6</v>
       </c>
       <c r="J276">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="K276" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="277" spans="1:11">
@@ -30081,25 +30081,25 @@
         <v>35</v>
       </c>
       <c r="E277">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F277">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G277" s="1">
-        <v>94.3</v>
+        <v>100</v>
       </c>
       <c r="H277" s="1">
-        <v>5.7</v>
+        <v>0</v>
       </c>
       <c r="I277" s="2">
-        <v>7.8</v>
+        <v>7.7</v>
       </c>
       <c r="J277">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="K277" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="278" spans="1:11">
@@ -30116,25 +30116,25 @@
         <v>24</v>
       </c>
       <c r="E278">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="F278">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="G278" s="1">
-        <v>83.3</v>
+        <v>100</v>
       </c>
       <c r="H278" s="1">
-        <v>16.7</v>
+        <v>0</v>
       </c>
       <c r="I278" s="2">
-        <v>7.5</v>
+        <v>7.4</v>
       </c>
       <c r="J278">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="K278" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="279" spans="1:11">
@@ -30148,25 +30148,25 @@
         <v>258</v>
       </c>
       <c r="E279">
-        <v>226</v>
+        <v>237</v>
       </c>
       <c r="F279">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="G279" s="1">
-        <v>87.59999999999999</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="H279" s="1">
-        <v>12.4</v>
+        <v>8.1</v>
       </c>
       <c r="I279" s="2">
         <v>7.9</v>
       </c>
       <c r="J279">
-        <v>258</v>
+        <v>118</v>
       </c>
       <c r="K279" s="1">
-        <v>100</v>
+        <v>45.7</v>
       </c>
     </row>
     <row r="280" spans="1:11">
@@ -30425,25 +30425,25 @@
         <v>22</v>
       </c>
       <c r="E287">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F287">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G287" s="1">
-        <v>68.2</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="H287" s="1">
-        <v>31.8</v>
+        <v>13.6</v>
       </c>
       <c r="I287" s="2">
-        <v>6.5</v>
+        <v>6.7</v>
       </c>
       <c r="J287">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="K287" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="288" spans="1:11">
@@ -30460,25 +30460,25 @@
         <v>29</v>
       </c>
       <c r="E288">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F288">
+        <v>0</v>
+      </c>
+      <c r="G288" s="1">
+        <v>96.59999999999999</v>
+      </c>
+      <c r="H288" s="1">
+        <v>0</v>
+      </c>
+      <c r="I288" s="2">
+        <v>8</v>
+      </c>
+      <c r="J288">
         <v>1</v>
       </c>
-      <c r="G288" s="1">
-        <v>93.09999999999999</v>
-      </c>
-      <c r="H288" s="1">
+      <c r="K288" s="1">
         <v>3.4</v>
-      </c>
-      <c r="I288" s="2">
-        <v>8.300000000000001</v>
-      </c>
-      <c r="J288">
-        <v>29</v>
-      </c>
-      <c r="K288" s="1">
-        <v>100</v>
       </c>
     </row>
     <row r="289" spans="1:11">
@@ -30495,25 +30495,25 @@
         <v>31</v>
       </c>
       <c r="E289">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F289">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G289" s="1">
-        <v>93.5</v>
+        <v>100</v>
       </c>
       <c r="H289" s="1">
-        <v>6.5</v>
+        <v>0</v>
       </c>
       <c r="I289" s="2">
         <v>7.8</v>
       </c>
       <c r="J289">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="K289" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="290" spans="1:11">
@@ -30597,25 +30597,25 @@
         <v>126</v>
       </c>
       <c r="E292">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="F292">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="G292" s="1">
-        <v>88.09999999999999</v>
+        <v>93.7</v>
       </c>
       <c r="H292" s="1">
-        <v>9.5</v>
+        <v>4</v>
       </c>
       <c r="I292" s="2">
         <v>7.6</v>
       </c>
       <c r="J292">
-        <v>126</v>
+        <v>45</v>
       </c>
       <c r="K292" s="1">
-        <v>100</v>
+        <v>35.7</v>
       </c>
     </row>
     <row r="293" spans="1:11">

</xml_diff>